<commit_message>
Add GMAC neural decoder results: BiGRU and MLP, N=8-1024
GMAC Class B, SNR=6dB, rho=0.7 (symmetric ku=kv).
BiGRU z_encoder: beats SC at N=8-32, ratio grows to 47x at N=1024.
Simple MLP z_encoder: beats SC at N=32, degrades faster at large N.
Key finding: MLP matches BiGRU at N<=128 (memoryless channel),
BiGRU wins at N>=256 due to richer codeword-level embeddings.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/gmac_snr6dB/gmac_snr6dB_classB_Ru48_Rv48_nn_vs_sc/nn_vs_sc_classB_Ru48_Rv48_snr6dB.xlsx
+++ b/results/gmac_snr6dB/gmac_snr6dB_classB_Ru48_Rv48_nn_vs_sc/nn_vs_sc_classB_Ru48_Rv48_snr6dB.xlsx
@@ -471,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:I14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -488,7 +488,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Gaussian MAC (6dB) — Class B, (Ru=0.48, Rv=0.48), Neural SC vs SC (L=1)</t>
+          <t>Gaussian MAC (6dB) — Class B, (Ru≈0.48, Rv≈0.48), Neural SC vs SC (L=1)</t>
         </is>
       </c>
     </row>
@@ -720,24 +720,82 @@
         <v>2000</v>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" s="4" t="n">
+        <v>512</v>
+      </c>
+      <c r="B11" s="4" t="n">
+        <v>247</v>
+      </c>
+      <c r="C11" s="4" t="n">
+        <v>247</v>
+      </c>
+      <c r="D11" s="5" t="n">
+        <v>0.482421875</v>
+      </c>
+      <c r="E11" s="5" t="n">
+        <v>0.482421875</v>
+      </c>
+      <c r="F11" s="6" t="n">
+        <v>0.019</v>
+      </c>
+      <c r="G11" s="6" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="H11" s="7" t="n">
+        <v>19</v>
+      </c>
+      <c r="I11" s="4" t="n">
+        <v>1000</v>
+      </c>
+    </row>
     <row r="12">
-      <c r="A12" s="8" t="inlineStr">
+      <c r="A12" s="4" t="n">
+        <v>1024</v>
+      </c>
+      <c r="B12" s="4" t="n">
+        <v>493</v>
+      </c>
+      <c r="C12" s="4" t="n">
+        <v>493</v>
+      </c>
+      <c r="D12" s="5" t="n">
+        <v>0.4814453125</v>
+      </c>
+      <c r="E12" s="5" t="n">
+        <v>0.4814453125</v>
+      </c>
+      <c r="F12" s="6" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="G12" s="6" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="H12" s="7" t="n">
+        <v>46.67</v>
+      </c>
+      <c r="I12" s="4" t="n">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr">
         <is>
           <t>Capacity</t>
         </is>
       </c>
-      <c r="B12" s="4" t="n"/>
-      <c r="C12" s="4" t="n"/>
-      <c r="D12" s="5" t="n">
+      <c r="B14" s="4" t="n"/>
+      <c r="C14" s="4" t="n"/>
+      <c r="D14" s="5" t="n">
         <v>0.688195269487774</v>
       </c>
-      <c r="E12" s="5" t="n">
+      <c r="E14" s="5" t="n">
         <v>0.688195269487774</v>
       </c>
-      <c r="F12" s="4" t="n"/>
-      <c r="G12" s="4" t="n"/>
-      <c r="H12" s="4" t="n"/>
-      <c r="I12" s="4" t="n"/>
+      <c r="F14" s="4" t="n"/>
+      <c r="G14" s="4" t="n"/>
+      <c r="H14" s="4" t="n"/>
+      <c r="I14" s="4" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
Update NN vs SC xlsx and plot with latest results (N=256: 0.015, N=512: 0.018)
Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/gmac_snr6dB/gmac_snr6dB_classB_Ru48_Rv48_nn_vs_sc/nn_vs_sc_classB_Ru48_Rv48_snr6dB.xlsx
+++ b/results/gmac_snr6dB/gmac_snr6dB_classB_Ru48_Rv48_nn_vs_sc/nn_vs_sc_classB_Ru48_Rv48_snr6dB.xlsx
@@ -566,7 +566,7 @@
         <v>0.037</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>0.07240000000000001</v>
+        <v>0.07199999999999999</v>
       </c>
       <c r="H5" s="7" t="n">
         <v>0.51</v>
@@ -595,7 +595,7 @@
         <v>0.06900000000000001</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>0.0638</v>
+        <v>0.064</v>
       </c>
       <c r="H6" s="7" t="n">
         <v>1.08</v>
@@ -621,16 +621,16 @@
         <v>0.46875</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>0.0444</v>
+        <v>0.046</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>0.0456</v>
+        <v>0.046</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>0.97</v>
+        <v>1</v>
       </c>
       <c r="I7" s="4" t="n">
-        <v>5000</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="8">
@@ -650,16 +650,16 @@
         <v>0.484375</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>0.0324</v>
+        <v>0.026</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>0.0246</v>
+        <v>0.025</v>
       </c>
       <c r="H8" s="7" t="n">
-        <v>1.32</v>
+        <v>1.04</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>5000</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="9">
@@ -679,13 +679,13 @@
         <v>0.484375</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>0.03266666666666666</v>
+        <v>0.017</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>0.01585</v>
+        <v>0.016</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>2.06</v>
+        <v>1.06</v>
       </c>
       <c r="I9" s="4" t="n">
         <v>3000</v>
@@ -708,16 +708,16 @@
         <v>0.48046875</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>0.0205</v>
+        <v>0.015</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>0.004567</v>
+        <v>0.005</v>
       </c>
       <c r="H10" s="7" t="n">
-        <v>4.49</v>
+        <v>3</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>10000</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="11">
@@ -737,16 +737,16 @@
         <v>0.482421875</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>0.019</v>
+        <v>0.018</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>0.00106</v>
+        <v>0.001</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>17.92</v>
+        <v>18</v>
       </c>
       <c r="I11" s="4" t="n">
-        <v>50000</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="12">
@@ -766,16 +766,16 @@
         <v>0.4814453125</v>
       </c>
       <c r="F12" s="6" t="n">
-        <v>0.014</v>
+        <v>0.06900000000000001</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>0.00102</v>
+        <v>0.001</v>
       </c>
       <c r="H12" s="7" t="n">
-        <v>13.73</v>
+        <v>69</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>50000</v>
+        <v>200</v>
       </c>
     </row>
     <row r="14">

</xml_diff>